<commit_message>
Post Processing Work Complete and functional
</commit_message>
<xml_diff>
--- a/app/process_data/df_final.audit.xlsx
+++ b/app/process_data/df_final.audit.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T249"/>
+  <dimension ref="A1:V249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,6 +524,16 @@
           <t>_score</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>ActualFPTS_Rank</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -596,6 +606,12 @@
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>9</v>
+      </c>
+      <c r="V2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -668,6 +684,12 @@
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>9</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -740,6 +762,12 @@
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
+      <c r="U4" t="n">
+        <v>9</v>
+      </c>
+      <c r="V4" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -812,6 +840,12 @@
         </is>
       </c>
       <c r="T5" t="inlineStr"/>
+      <c r="U5" t="n">
+        <v>9</v>
+      </c>
+      <c r="V5" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -884,6 +918,12 @@
         </is>
       </c>
       <c r="T6" t="inlineStr"/>
+      <c r="U6" t="n">
+        <v>9</v>
+      </c>
+      <c r="V6" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -956,6 +996,12 @@
         </is>
       </c>
       <c r="T7" t="inlineStr"/>
+      <c r="U7" t="n">
+        <v>9</v>
+      </c>
+      <c r="V7" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1028,6 +1074,12 @@
         </is>
       </c>
       <c r="T8" t="inlineStr"/>
+      <c r="U8" t="n">
+        <v>9</v>
+      </c>
+      <c r="V8" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -1100,6 +1152,12 @@
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
+      <c r="U9" t="n">
+        <v>9</v>
+      </c>
+      <c r="V9" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -1172,6 +1230,12 @@
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
+      <c r="U10" t="n">
+        <v>9</v>
+      </c>
+      <c r="V10" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1244,6 +1308,12 @@
         </is>
       </c>
       <c r="T11" t="inlineStr"/>
+      <c r="U11" t="n">
+        <v>9</v>
+      </c>
+      <c r="V11" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -1316,6 +1386,12 @@
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
+      <c r="U12" t="n">
+        <v>9</v>
+      </c>
+      <c r="V12" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -1388,6 +1464,12 @@
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
+      <c r="U13" t="n">
+        <v>9</v>
+      </c>
+      <c r="V13" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -1460,6 +1542,12 @@
         </is>
       </c>
       <c r="T14" t="inlineStr"/>
+      <c r="U14" t="n">
+        <v>9</v>
+      </c>
+      <c r="V14" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1532,6 +1620,12 @@
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
+      <c r="U15" t="n">
+        <v>9</v>
+      </c>
+      <c r="V15" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -1604,6 +1698,12 @@
         </is>
       </c>
       <c r="T16" t="inlineStr"/>
+      <c r="U16" t="n">
+        <v>9</v>
+      </c>
+      <c r="V16" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -1676,6 +1776,12 @@
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
+      <c r="U17" t="n">
+        <v>9</v>
+      </c>
+      <c r="V17" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -1748,6 +1854,12 @@
         </is>
       </c>
       <c r="T18" t="inlineStr"/>
+      <c r="U18" t="n">
+        <v>9</v>
+      </c>
+      <c r="V18" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -1820,6 +1932,12 @@
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
+      <c r="U19" t="n">
+        <v>9</v>
+      </c>
+      <c r="V19" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -1892,6 +2010,12 @@
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
+      <c r="U20" t="n">
+        <v>9</v>
+      </c>
+      <c r="V20" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -1964,6 +2088,12 @@
         </is>
       </c>
       <c r="T21" t="inlineStr"/>
+      <c r="U21" t="n">
+        <v>9</v>
+      </c>
+      <c r="V21" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -2036,6 +2166,12 @@
         </is>
       </c>
       <c r="T22" t="inlineStr"/>
+      <c r="U22" t="n">
+        <v>9</v>
+      </c>
+      <c r="V22" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -2108,6 +2244,12 @@
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
+      <c r="U23" t="n">
+        <v>9</v>
+      </c>
+      <c r="V23" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -2180,6 +2322,12 @@
         </is>
       </c>
       <c r="T24" t="inlineStr"/>
+      <c r="U24" t="n">
+        <v>9</v>
+      </c>
+      <c r="V24" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -2252,6 +2400,12 @@
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
+      <c r="U25" t="n">
+        <v>9</v>
+      </c>
+      <c r="V25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -2324,6 +2478,12 @@
         </is>
       </c>
       <c r="T26" t="inlineStr"/>
+      <c r="U26" t="n">
+        <v>9</v>
+      </c>
+      <c r="V26" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -2396,6 +2556,12 @@
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
+      <c r="U27" t="n">
+        <v>9</v>
+      </c>
+      <c r="V27" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -2468,6 +2634,12 @@
         </is>
       </c>
       <c r="T28" t="inlineStr"/>
+      <c r="U28" t="n">
+        <v>9</v>
+      </c>
+      <c r="V28" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -2540,6 +2712,12 @@
         </is>
       </c>
       <c r="T29" t="inlineStr"/>
+      <c r="U29" t="n">
+        <v>9</v>
+      </c>
+      <c r="V29" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -2612,6 +2790,12 @@
         </is>
       </c>
       <c r="T30" t="inlineStr"/>
+      <c r="U30" t="n">
+        <v>9</v>
+      </c>
+      <c r="V30" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -2684,6 +2868,12 @@
         </is>
       </c>
       <c r="T31" t="inlineStr"/>
+      <c r="U31" t="n">
+        <v>9</v>
+      </c>
+      <c r="V31" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -2756,6 +2946,12 @@
         </is>
       </c>
       <c r="T32" t="inlineStr"/>
+      <c r="U32" t="n">
+        <v>9</v>
+      </c>
+      <c r="V32" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -2828,6 +3024,12 @@
         </is>
       </c>
       <c r="T33" t="inlineStr"/>
+      <c r="U33" t="n">
+        <v>9</v>
+      </c>
+      <c r="V33" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -2900,6 +3102,12 @@
         </is>
       </c>
       <c r="T34" t="inlineStr"/>
+      <c r="U34" t="n">
+        <v>9</v>
+      </c>
+      <c r="V34" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -2972,6 +3180,12 @@
         </is>
       </c>
       <c r="T35" t="inlineStr"/>
+      <c r="U35" t="n">
+        <v>9</v>
+      </c>
+      <c r="V35" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -3044,6 +3258,12 @@
         </is>
       </c>
       <c r="T36" t="inlineStr"/>
+      <c r="U36" t="n">
+        <v>9</v>
+      </c>
+      <c r="V36" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -3116,6 +3336,12 @@
         </is>
       </c>
       <c r="T37" t="inlineStr"/>
+      <c r="U37" t="n">
+        <v>9</v>
+      </c>
+      <c r="V37" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -3188,6 +3414,12 @@
         </is>
       </c>
       <c r="T38" t="inlineStr"/>
+      <c r="U38" t="n">
+        <v>9</v>
+      </c>
+      <c r="V38" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -3260,6 +3492,12 @@
         </is>
       </c>
       <c r="T39" t="inlineStr"/>
+      <c r="U39" t="n">
+        <v>9</v>
+      </c>
+      <c r="V39" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -3332,6 +3570,12 @@
         </is>
       </c>
       <c r="T40" t="inlineStr"/>
+      <c r="U40" t="n">
+        <v>9</v>
+      </c>
+      <c r="V40" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -3404,6 +3648,12 @@
         </is>
       </c>
       <c r="T41" t="inlineStr"/>
+      <c r="U41" t="n">
+        <v>9</v>
+      </c>
+      <c r="V41" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -3476,6 +3726,12 @@
         </is>
       </c>
       <c r="T42" t="inlineStr"/>
+      <c r="U42" t="n">
+        <v>9</v>
+      </c>
+      <c r="V42" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
@@ -3548,6 +3804,12 @@
         </is>
       </c>
       <c r="T43" t="inlineStr"/>
+      <c r="U43" t="n">
+        <v>9</v>
+      </c>
+      <c r="V43" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
@@ -3620,6 +3882,12 @@
         </is>
       </c>
       <c r="T44" t="inlineStr"/>
+      <c r="U44" t="n">
+        <v>9</v>
+      </c>
+      <c r="V44" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
@@ -3692,6 +3960,12 @@
         </is>
       </c>
       <c r="T45" t="inlineStr"/>
+      <c r="U45" t="n">
+        <v>9</v>
+      </c>
+      <c r="V45" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
@@ -3764,6 +4038,12 @@
         </is>
       </c>
       <c r="T46" t="inlineStr"/>
+      <c r="U46" t="n">
+        <v>9</v>
+      </c>
+      <c r="V46" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
@@ -3836,6 +4116,12 @@
         </is>
       </c>
       <c r="T47" t="inlineStr"/>
+      <c r="U47" t="n">
+        <v>9</v>
+      </c>
+      <c r="V47" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -3908,6 +4194,12 @@
         </is>
       </c>
       <c r="T48" t="inlineStr"/>
+      <c r="U48" t="n">
+        <v>9</v>
+      </c>
+      <c r="V48" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -3980,6 +4272,12 @@
         </is>
       </c>
       <c r="T49" t="inlineStr"/>
+      <c r="U49" t="n">
+        <v>9</v>
+      </c>
+      <c r="V49" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -4052,6 +4350,12 @@
         </is>
       </c>
       <c r="T50" t="inlineStr"/>
+      <c r="U50" t="n">
+        <v>9</v>
+      </c>
+      <c r="V50" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -4124,6 +4428,12 @@
         </is>
       </c>
       <c r="T51" t="inlineStr"/>
+      <c r="U51" t="n">
+        <v>9</v>
+      </c>
+      <c r="V51" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -4196,6 +4506,12 @@
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
+      <c r="U52" t="n">
+        <v>9</v>
+      </c>
+      <c r="V52" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -4268,6 +4584,12 @@
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
+      <c r="U53" t="n">
+        <v>9</v>
+      </c>
+      <c r="V53" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -4340,6 +4662,12 @@
         </is>
       </c>
       <c r="T54" t="inlineStr"/>
+      <c r="U54" t="n">
+        <v>9</v>
+      </c>
+      <c r="V54" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -4412,6 +4740,12 @@
         </is>
       </c>
       <c r="T55" t="inlineStr"/>
+      <c r="U55" t="n">
+        <v>9</v>
+      </c>
+      <c r="V55" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
@@ -4484,6 +4818,12 @@
         </is>
       </c>
       <c r="T56" t="inlineStr"/>
+      <c r="U56" t="n">
+        <v>9</v>
+      </c>
+      <c r="V56" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
@@ -4556,6 +4896,12 @@
         </is>
       </c>
       <c r="T57" t="inlineStr"/>
+      <c r="U57" t="n">
+        <v>9</v>
+      </c>
+      <c r="V57" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
@@ -4628,6 +4974,12 @@
         </is>
       </c>
       <c r="T58" t="inlineStr"/>
+      <c r="U58" t="n">
+        <v>9</v>
+      </c>
+      <c r="V58" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
@@ -4700,6 +5052,12 @@
         </is>
       </c>
       <c r="T59" t="inlineStr"/>
+      <c r="U59" t="n">
+        <v>9</v>
+      </c>
+      <c r="V59" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
@@ -4772,6 +5130,12 @@
         </is>
       </c>
       <c r="T60" t="inlineStr"/>
+      <c r="U60" t="n">
+        <v>9</v>
+      </c>
+      <c r="V60" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
@@ -4844,6 +5208,12 @@
         </is>
       </c>
       <c r="T61" t="inlineStr"/>
+      <c r="U61" t="n">
+        <v>9</v>
+      </c>
+      <c r="V61" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
@@ -4916,6 +5286,12 @@
         </is>
       </c>
       <c r="T62" t="inlineStr"/>
+      <c r="U62" t="n">
+        <v>9</v>
+      </c>
+      <c r="V62" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -4988,6 +5364,12 @@
         </is>
       </c>
       <c r="T63" t="inlineStr"/>
+      <c r="U63" t="n">
+        <v>9</v>
+      </c>
+      <c r="V63" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
@@ -5060,6 +5442,12 @@
         </is>
       </c>
       <c r="T64" t="inlineStr"/>
+      <c r="U64" t="n">
+        <v>9</v>
+      </c>
+      <c r="V64" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -5132,6 +5520,12 @@
         </is>
       </c>
       <c r="T65" t="inlineStr"/>
+      <c r="U65" t="n">
+        <v>9</v>
+      </c>
+      <c r="V65" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
@@ -5204,6 +5598,12 @@
         </is>
       </c>
       <c r="T66" t="inlineStr"/>
+      <c r="U66" t="n">
+        <v>9</v>
+      </c>
+      <c r="V66" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
@@ -5276,6 +5676,12 @@
         </is>
       </c>
       <c r="T67" t="inlineStr"/>
+      <c r="U67" t="n">
+        <v>9</v>
+      </c>
+      <c r="V67" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
@@ -5348,6 +5754,12 @@
         </is>
       </c>
       <c r="T68" t="inlineStr"/>
+      <c r="U68" t="n">
+        <v>9</v>
+      </c>
+      <c r="V68" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
@@ -5420,6 +5832,12 @@
         </is>
       </c>
       <c r="T69" t="inlineStr"/>
+      <c r="U69" t="n">
+        <v>9</v>
+      </c>
+      <c r="V69" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
@@ -5492,6 +5910,12 @@
         </is>
       </c>
       <c r="T70" t="inlineStr"/>
+      <c r="U70" t="n">
+        <v>9</v>
+      </c>
+      <c r="V70" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
@@ -5564,6 +5988,12 @@
         </is>
       </c>
       <c r="T71" t="inlineStr"/>
+      <c r="U71" t="n">
+        <v>9</v>
+      </c>
+      <c r="V71" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
@@ -5636,6 +6066,12 @@
         </is>
       </c>
       <c r="T72" t="inlineStr"/>
+      <c r="U72" t="n">
+        <v>9</v>
+      </c>
+      <c r="V72" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
@@ -5708,6 +6144,12 @@
         </is>
       </c>
       <c r="T73" t="inlineStr"/>
+      <c r="U73" t="n">
+        <v>9</v>
+      </c>
+      <c r="V73" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
@@ -5780,6 +6222,12 @@
         </is>
       </c>
       <c r="T74" t="inlineStr"/>
+      <c r="U74" t="n">
+        <v>9</v>
+      </c>
+      <c r="V74" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
@@ -5852,6 +6300,12 @@
         </is>
       </c>
       <c r="T75" t="inlineStr"/>
+      <c r="U75" t="n">
+        <v>9</v>
+      </c>
+      <c r="V75" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
@@ -5924,6 +6378,12 @@
         </is>
       </c>
       <c r="T76" t="inlineStr"/>
+      <c r="U76" t="n">
+        <v>9</v>
+      </c>
+      <c r="V76" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
@@ -5996,6 +6456,12 @@
         </is>
       </c>
       <c r="T77" t="inlineStr"/>
+      <c r="U77" t="n">
+        <v>9</v>
+      </c>
+      <c r="V77" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
@@ -6068,6 +6534,12 @@
         </is>
       </c>
       <c r="T78" t="inlineStr"/>
+      <c r="U78" t="n">
+        <v>9</v>
+      </c>
+      <c r="V78" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
@@ -6140,6 +6612,12 @@
         </is>
       </c>
       <c r="T79" t="inlineStr"/>
+      <c r="U79" t="n">
+        <v>9</v>
+      </c>
+      <c r="V79" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
@@ -6212,6 +6690,12 @@
         </is>
       </c>
       <c r="T80" t="inlineStr"/>
+      <c r="U80" t="n">
+        <v>9</v>
+      </c>
+      <c r="V80" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
@@ -6284,6 +6768,12 @@
         </is>
       </c>
       <c r="T81" t="inlineStr"/>
+      <c r="U81" t="n">
+        <v>9</v>
+      </c>
+      <c r="V81" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
@@ -6356,6 +6846,12 @@
         </is>
       </c>
       <c r="T82" t="inlineStr"/>
+      <c r="U82" t="n">
+        <v>9</v>
+      </c>
+      <c r="V82" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -6428,6 +6924,12 @@
         </is>
       </c>
       <c r="T83" t="inlineStr"/>
+      <c r="U83" t="n">
+        <v>9</v>
+      </c>
+      <c r="V83" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
@@ -6500,6 +7002,12 @@
         </is>
       </c>
       <c r="T84" t="inlineStr"/>
+      <c r="U84" t="n">
+        <v>9</v>
+      </c>
+      <c r="V84" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
@@ -6572,6 +7080,12 @@
         </is>
       </c>
       <c r="T85" t="inlineStr"/>
+      <c r="U85" t="n">
+        <v>9</v>
+      </c>
+      <c r="V85" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
@@ -6644,6 +7158,12 @@
         </is>
       </c>
       <c r="T86" t="inlineStr"/>
+      <c r="U86" t="n">
+        <v>9</v>
+      </c>
+      <c r="V86" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
@@ -6716,6 +7236,12 @@
         </is>
       </c>
       <c r="T87" t="inlineStr"/>
+      <c r="U87" t="n">
+        <v>9</v>
+      </c>
+      <c r="V87" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
@@ -6788,6 +7314,12 @@
         </is>
       </c>
       <c r="T88" t="inlineStr"/>
+      <c r="U88" t="n">
+        <v>9</v>
+      </c>
+      <c r="V88" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
@@ -6860,6 +7392,12 @@
         </is>
       </c>
       <c r="T89" t="inlineStr"/>
+      <c r="U89" t="n">
+        <v>9</v>
+      </c>
+      <c r="V89" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
@@ -6932,6 +7470,12 @@
         </is>
       </c>
       <c r="T90" t="inlineStr"/>
+      <c r="U90" t="n">
+        <v>9</v>
+      </c>
+      <c r="V90" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
@@ -7004,6 +7548,12 @@
         </is>
       </c>
       <c r="T91" t="inlineStr"/>
+      <c r="U91" t="n">
+        <v>9</v>
+      </c>
+      <c r="V91" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
@@ -7076,6 +7626,12 @@
         </is>
       </c>
       <c r="T92" t="inlineStr"/>
+      <c r="U92" t="n">
+        <v>9</v>
+      </c>
+      <c r="V92" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
@@ -7148,6 +7704,12 @@
         </is>
       </c>
       <c r="T93" t="inlineStr"/>
+      <c r="U93" t="n">
+        <v>9</v>
+      </c>
+      <c r="V93" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -7220,6 +7782,12 @@
         </is>
       </c>
       <c r="T94" t="inlineStr"/>
+      <c r="U94" t="n">
+        <v>9</v>
+      </c>
+      <c r="V94" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
@@ -7292,6 +7860,12 @@
         </is>
       </c>
       <c r="T95" t="inlineStr"/>
+      <c r="U95" t="n">
+        <v>9</v>
+      </c>
+      <c r="V95" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
@@ -7364,6 +7938,12 @@
         </is>
       </c>
       <c r="T96" t="inlineStr"/>
+      <c r="U96" t="n">
+        <v>9</v>
+      </c>
+      <c r="V96" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
@@ -7436,6 +8016,12 @@
         </is>
       </c>
       <c r="T97" t="inlineStr"/>
+      <c r="U97" t="n">
+        <v>9</v>
+      </c>
+      <c r="V97" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
@@ -7508,6 +8094,12 @@
         </is>
       </c>
       <c r="T98" t="inlineStr"/>
+      <c r="U98" t="n">
+        <v>9</v>
+      </c>
+      <c r="V98" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
@@ -7580,6 +8172,12 @@
         </is>
       </c>
       <c r="T99" t="inlineStr"/>
+      <c r="U99" t="n">
+        <v>9</v>
+      </c>
+      <c r="V99" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
@@ -7652,6 +8250,12 @@
         </is>
       </c>
       <c r="T100" t="inlineStr"/>
+      <c r="U100" t="n">
+        <v>9</v>
+      </c>
+      <c r="V100" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
@@ -7724,6 +8328,12 @@
         </is>
       </c>
       <c r="T101" t="inlineStr"/>
+      <c r="U101" t="n">
+        <v>9</v>
+      </c>
+      <c r="V101" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
@@ -7796,6 +8406,12 @@
         </is>
       </c>
       <c r="T102" t="inlineStr"/>
+      <c r="U102" t="n">
+        <v>9</v>
+      </c>
+      <c r="V102" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
@@ -7868,6 +8484,12 @@
         </is>
       </c>
       <c r="T103" t="inlineStr"/>
+      <c r="U103" t="n">
+        <v>9</v>
+      </c>
+      <c r="V103" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
@@ -7940,6 +8562,12 @@
         </is>
       </c>
       <c r="T104" t="inlineStr"/>
+      <c r="U104" t="n">
+        <v>9</v>
+      </c>
+      <c r="V104" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -8012,6 +8640,12 @@
         </is>
       </c>
       <c r="T105" t="inlineStr"/>
+      <c r="U105" t="n">
+        <v>9</v>
+      </c>
+      <c r="V105" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
@@ -8084,6 +8718,12 @@
         </is>
       </c>
       <c r="T106" t="inlineStr"/>
+      <c r="U106" t="n">
+        <v>9</v>
+      </c>
+      <c r="V106" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
@@ -8156,6 +8796,12 @@
         </is>
       </c>
       <c r="T107" t="inlineStr"/>
+      <c r="U107" t="n">
+        <v>9</v>
+      </c>
+      <c r="V107" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
@@ -8228,6 +8874,12 @@
         </is>
       </c>
       <c r="T108" t="inlineStr"/>
+      <c r="U108" t="n">
+        <v>9</v>
+      </c>
+      <c r="V108" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
@@ -8300,6 +8952,12 @@
         </is>
       </c>
       <c r="T109" t="inlineStr"/>
+      <c r="U109" t="n">
+        <v>9</v>
+      </c>
+      <c r="V109" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
@@ -8372,6 +9030,12 @@
         </is>
       </c>
       <c r="T110" t="inlineStr"/>
+      <c r="U110" t="n">
+        <v>9</v>
+      </c>
+      <c r="V110" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
@@ -8444,6 +9108,12 @@
         </is>
       </c>
       <c r="T111" t="inlineStr"/>
+      <c r="U111" t="n">
+        <v>9</v>
+      </c>
+      <c r="V111" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
@@ -8516,6 +9186,12 @@
         </is>
       </c>
       <c r="T112" t="inlineStr"/>
+      <c r="U112" t="n">
+        <v>9</v>
+      </c>
+      <c r="V112" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
@@ -8588,6 +9264,12 @@
         </is>
       </c>
       <c r="T113" t="inlineStr"/>
+      <c r="U113" t="n">
+        <v>9</v>
+      </c>
+      <c r="V113" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
@@ -8660,6 +9342,12 @@
         </is>
       </c>
       <c r="T114" t="inlineStr"/>
+      <c r="U114" t="n">
+        <v>9</v>
+      </c>
+      <c r="V114" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
@@ -8732,6 +9420,12 @@
         </is>
       </c>
       <c r="T115" t="inlineStr"/>
+      <c r="U115" t="n">
+        <v>9</v>
+      </c>
+      <c r="V115" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
@@ -8804,6 +9498,12 @@
         </is>
       </c>
       <c r="T116" t="inlineStr"/>
+      <c r="U116" t="n">
+        <v>9</v>
+      </c>
+      <c r="V116" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
@@ -8876,6 +9576,12 @@
         </is>
       </c>
       <c r="T117" t="inlineStr"/>
+      <c r="U117" t="n">
+        <v>9</v>
+      </c>
+      <c r="V117" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
@@ -8948,6 +9654,12 @@
         </is>
       </c>
       <c r="T118" t="inlineStr"/>
+      <c r="U118" t="n">
+        <v>9</v>
+      </c>
+      <c r="V118" t="n">
+        <v>72</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
@@ -9020,6 +9732,12 @@
         </is>
       </c>
       <c r="T119" t="inlineStr"/>
+      <c r="U119" t="n">
+        <v>9</v>
+      </c>
+      <c r="V119" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
@@ -9092,6 +9810,12 @@
         </is>
       </c>
       <c r="T120" t="inlineStr"/>
+      <c r="U120" t="n">
+        <v>9</v>
+      </c>
+      <c r="V120" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
@@ -9164,6 +9888,12 @@
         </is>
       </c>
       <c r="T121" t="inlineStr"/>
+      <c r="U121" t="n">
+        <v>9</v>
+      </c>
+      <c r="V121" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
@@ -9236,6 +9966,12 @@
         </is>
       </c>
       <c r="T122" t="inlineStr"/>
+      <c r="U122" t="n">
+        <v>9</v>
+      </c>
+      <c r="V122" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
@@ -9308,6 +10044,12 @@
         </is>
       </c>
       <c r="T123" t="inlineStr"/>
+      <c r="U123" t="n">
+        <v>9</v>
+      </c>
+      <c r="V123" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
@@ -9380,6 +10122,12 @@
         </is>
       </c>
       <c r="T124" t="inlineStr"/>
+      <c r="U124" t="n">
+        <v>9</v>
+      </c>
+      <c r="V124" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
@@ -9452,6 +10200,12 @@
         </is>
       </c>
       <c r="T125" t="inlineStr"/>
+      <c r="U125" t="n">
+        <v>9</v>
+      </c>
+      <c r="V125" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
@@ -9524,6 +10278,12 @@
         </is>
       </c>
       <c r="T126" t="inlineStr"/>
+      <c r="U126" t="n">
+        <v>9</v>
+      </c>
+      <c r="V126" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
@@ -9596,6 +10356,12 @@
         </is>
       </c>
       <c r="T127" t="inlineStr"/>
+      <c r="U127" t="n">
+        <v>9</v>
+      </c>
+      <c r="V127" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
@@ -9668,6 +10434,12 @@
         </is>
       </c>
       <c r="T128" t="inlineStr"/>
+      <c r="U128" t="n">
+        <v>9</v>
+      </c>
+      <c r="V128" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
@@ -9740,6 +10512,12 @@
         </is>
       </c>
       <c r="T129" t="inlineStr"/>
+      <c r="U129" t="n">
+        <v>9</v>
+      </c>
+      <c r="V129" t="n">
+        <v>71</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
@@ -9812,6 +10590,12 @@
         </is>
       </c>
       <c r="T130" t="inlineStr"/>
+      <c r="U130" t="n">
+        <v>9</v>
+      </c>
+      <c r="V130" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
@@ -9884,6 +10668,12 @@
         </is>
       </c>
       <c r="T131" t="inlineStr"/>
+      <c r="U131" t="n">
+        <v>9</v>
+      </c>
+      <c r="V131" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
@@ -9956,6 +10746,12 @@
         </is>
       </c>
       <c r="T132" t="inlineStr"/>
+      <c r="U132" t="n">
+        <v>9</v>
+      </c>
+      <c r="V132" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
@@ -10028,6 +10824,12 @@
         </is>
       </c>
       <c r="T133" t="inlineStr"/>
+      <c r="U133" t="n">
+        <v>9</v>
+      </c>
+      <c r="V133" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
@@ -10100,6 +10902,12 @@
         </is>
       </c>
       <c r="T134" t="inlineStr"/>
+      <c r="U134" t="n">
+        <v>9</v>
+      </c>
+      <c r="V134" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
@@ -10172,6 +10980,12 @@
         </is>
       </c>
       <c r="T135" t="inlineStr"/>
+      <c r="U135" t="n">
+        <v>9</v>
+      </c>
+      <c r="V135" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
@@ -10244,6 +11058,12 @@
         </is>
       </c>
       <c r="T136" t="inlineStr"/>
+      <c r="U136" t="n">
+        <v>9</v>
+      </c>
+      <c r="V136" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
@@ -10316,6 +11136,12 @@
         </is>
       </c>
       <c r="T137" t="inlineStr"/>
+      <c r="U137" t="n">
+        <v>9</v>
+      </c>
+      <c r="V137" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
@@ -10388,6 +11214,12 @@
         </is>
       </c>
       <c r="T138" t="inlineStr"/>
+      <c r="U138" t="n">
+        <v>9</v>
+      </c>
+      <c r="V138" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
@@ -10460,6 +11292,12 @@
         </is>
       </c>
       <c r="T139" t="inlineStr"/>
+      <c r="U139" t="n">
+        <v>9</v>
+      </c>
+      <c r="V139" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
@@ -10532,6 +11370,12 @@
         </is>
       </c>
       <c r="T140" t="inlineStr"/>
+      <c r="U140" t="n">
+        <v>9</v>
+      </c>
+      <c r="V140" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
@@ -10604,6 +11448,12 @@
         </is>
       </c>
       <c r="T141" t="inlineStr"/>
+      <c r="U141" t="n">
+        <v>9</v>
+      </c>
+      <c r="V141" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
@@ -10676,6 +11526,12 @@
         </is>
       </c>
       <c r="T142" t="inlineStr"/>
+      <c r="U142" t="n">
+        <v>9</v>
+      </c>
+      <c r="V142" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
@@ -10748,6 +11604,12 @@
         </is>
       </c>
       <c r="T143" t="inlineStr"/>
+      <c r="U143" t="n">
+        <v>9</v>
+      </c>
+      <c r="V143" t="n">
+        <v>64</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
@@ -10820,6 +11682,12 @@
         </is>
       </c>
       <c r="T144" t="inlineStr"/>
+      <c r="U144" t="n">
+        <v>9</v>
+      </c>
+      <c r="V144" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
@@ -10892,6 +11760,12 @@
         </is>
       </c>
       <c r="T145" t="inlineStr"/>
+      <c r="U145" t="n">
+        <v>9</v>
+      </c>
+      <c r="V145" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n">
@@ -10964,6 +11838,12 @@
         </is>
       </c>
       <c r="T146" t="inlineStr"/>
+      <c r="U146" t="n">
+        <v>9</v>
+      </c>
+      <c r="V146" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n">
@@ -11036,6 +11916,12 @@
         </is>
       </c>
       <c r="T147" t="inlineStr"/>
+      <c r="U147" t="n">
+        <v>9</v>
+      </c>
+      <c r="V147" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n">
@@ -11108,6 +11994,12 @@
         </is>
       </c>
       <c r="T148" t="inlineStr"/>
+      <c r="U148" t="n">
+        <v>9</v>
+      </c>
+      <c r="V148" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n">
@@ -11180,6 +12072,12 @@
         </is>
       </c>
       <c r="T149" t="inlineStr"/>
+      <c r="U149" t="n">
+        <v>9</v>
+      </c>
+      <c r="V149" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n">
@@ -11252,6 +12150,12 @@
         </is>
       </c>
       <c r="T150" t="inlineStr"/>
+      <c r="U150" t="n">
+        <v>9</v>
+      </c>
+      <c r="V150" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n">
@@ -11324,6 +12228,12 @@
         </is>
       </c>
       <c r="T151" t="inlineStr"/>
+      <c r="U151" t="n">
+        <v>9</v>
+      </c>
+      <c r="V151" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n">
@@ -11396,6 +12306,12 @@
         </is>
       </c>
       <c r="T152" t="inlineStr"/>
+      <c r="U152" t="n">
+        <v>9</v>
+      </c>
+      <c r="V152" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n">
@@ -11468,6 +12384,12 @@
         </is>
       </c>
       <c r="T153" t="inlineStr"/>
+      <c r="U153" t="n">
+        <v>9</v>
+      </c>
+      <c r="V153" t="n">
+        <v>54</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n">
@@ -11540,6 +12462,12 @@
         </is>
       </c>
       <c r="T154" t="inlineStr"/>
+      <c r="U154" t="n">
+        <v>9</v>
+      </c>
+      <c r="V154" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n">
@@ -11612,6 +12540,12 @@
         </is>
       </c>
       <c r="T155" t="inlineStr"/>
+      <c r="U155" t="n">
+        <v>9</v>
+      </c>
+      <c r="V155" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n">
@@ -11684,6 +12618,12 @@
         </is>
       </c>
       <c r="T156" t="inlineStr"/>
+      <c r="U156" t="n">
+        <v>9</v>
+      </c>
+      <c r="V156" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n">
@@ -11756,6 +12696,12 @@
         </is>
       </c>
       <c r="T157" t="inlineStr"/>
+      <c r="U157" t="n">
+        <v>9</v>
+      </c>
+      <c r="V157" t="n">
+        <v>95</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n">
@@ -11828,6 +12774,12 @@
         </is>
       </c>
       <c r="T158" t="inlineStr"/>
+      <c r="U158" t="n">
+        <v>9</v>
+      </c>
+      <c r="V158" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n">
@@ -11900,6 +12852,12 @@
         </is>
       </c>
       <c r="T159" t="inlineStr"/>
+      <c r="U159" t="n">
+        <v>9</v>
+      </c>
+      <c r="V159" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n">
@@ -11972,6 +12930,12 @@
         </is>
       </c>
       <c r="T160" t="inlineStr"/>
+      <c r="U160" t="n">
+        <v>9</v>
+      </c>
+      <c r="V160" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n">
@@ -12044,6 +13008,12 @@
         </is>
       </c>
       <c r="T161" t="inlineStr"/>
+      <c r="U161" t="n">
+        <v>9</v>
+      </c>
+      <c r="V161" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n">
@@ -12116,6 +13086,12 @@
         </is>
       </c>
       <c r="T162" t="inlineStr"/>
+      <c r="U162" t="n">
+        <v>9</v>
+      </c>
+      <c r="V162" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
@@ -12188,6 +13164,12 @@
         </is>
       </c>
       <c r="T163" t="inlineStr"/>
+      <c r="U163" t="n">
+        <v>9</v>
+      </c>
+      <c r="V163" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n">
@@ -12260,6 +13242,12 @@
         </is>
       </c>
       <c r="T164" t="inlineStr"/>
+      <c r="U164" t="n">
+        <v>9</v>
+      </c>
+      <c r="V164" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
@@ -12332,6 +13320,12 @@
         </is>
       </c>
       <c r="T165" t="inlineStr"/>
+      <c r="U165" t="n">
+        <v>9</v>
+      </c>
+      <c r="V165" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="n">
@@ -12404,6 +13398,12 @@
         </is>
       </c>
       <c r="T166" t="inlineStr"/>
+      <c r="U166" t="n">
+        <v>9</v>
+      </c>
+      <c r="V166" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
@@ -12476,6 +13476,12 @@
         </is>
       </c>
       <c r="T167" t="inlineStr"/>
+      <c r="U167" t="n">
+        <v>9</v>
+      </c>
+      <c r="V167" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
@@ -12548,6 +13554,12 @@
         </is>
       </c>
       <c r="T168" t="inlineStr"/>
+      <c r="U168" t="n">
+        <v>9</v>
+      </c>
+      <c r="V168" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n">
@@ -12620,6 +13632,12 @@
         </is>
       </c>
       <c r="T169" t="inlineStr"/>
+      <c r="U169" t="n">
+        <v>9</v>
+      </c>
+      <c r="V169" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n">
@@ -12692,6 +13710,12 @@
         </is>
       </c>
       <c r="T170" t="inlineStr"/>
+      <c r="U170" t="n">
+        <v>9</v>
+      </c>
+      <c r="V170" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="n">
@@ -12764,6 +13788,12 @@
         </is>
       </c>
       <c r="T171" t="inlineStr"/>
+      <c r="U171" t="n">
+        <v>9</v>
+      </c>
+      <c r="V171" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n">
@@ -12836,6 +13866,12 @@
         </is>
       </c>
       <c r="T172" t="inlineStr"/>
+      <c r="U172" t="n">
+        <v>9</v>
+      </c>
+      <c r="V172" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
@@ -12908,6 +13944,12 @@
         </is>
       </c>
       <c r="T173" t="inlineStr"/>
+      <c r="U173" t="n">
+        <v>9</v>
+      </c>
+      <c r="V173" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
@@ -12980,6 +14022,12 @@
         </is>
       </c>
       <c r="T174" t="inlineStr"/>
+      <c r="U174" t="n">
+        <v>9</v>
+      </c>
+      <c r="V174" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n">
@@ -13052,6 +14100,12 @@
         </is>
       </c>
       <c r="T175" t="inlineStr"/>
+      <c r="U175" t="n">
+        <v>9</v>
+      </c>
+      <c r="V175" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="n">
@@ -13124,6 +14178,12 @@
         </is>
       </c>
       <c r="T176" t="inlineStr"/>
+      <c r="U176" t="n">
+        <v>9</v>
+      </c>
+      <c r="V176" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n">
@@ -13196,6 +14256,12 @@
         </is>
       </c>
       <c r="T177" t="inlineStr"/>
+      <c r="U177" t="n">
+        <v>9</v>
+      </c>
+      <c r="V177" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
@@ -13268,6 +14334,12 @@
         </is>
       </c>
       <c r="T178" t="inlineStr"/>
+      <c r="U178" t="n">
+        <v>9</v>
+      </c>
+      <c r="V178" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n">
@@ -13340,6 +14412,12 @@
         </is>
       </c>
       <c r="T179" t="inlineStr"/>
+      <c r="U179" t="n">
+        <v>9</v>
+      </c>
+      <c r="V179" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n">
@@ -13412,6 +14490,12 @@
         </is>
       </c>
       <c r="T180" t="inlineStr"/>
+      <c r="U180" t="n">
+        <v>9</v>
+      </c>
+      <c r="V180" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n">
@@ -13484,6 +14568,12 @@
         </is>
       </c>
       <c r="T181" t="inlineStr"/>
+      <c r="U181" t="n">
+        <v>9</v>
+      </c>
+      <c r="V181" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="n">
@@ -13556,6 +14646,12 @@
         </is>
       </c>
       <c r="T182" t="inlineStr"/>
+      <c r="U182" t="n">
+        <v>9</v>
+      </c>
+      <c r="V182" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="n">
@@ -13628,6 +14724,12 @@
         </is>
       </c>
       <c r="T183" t="inlineStr"/>
+      <c r="U183" t="n">
+        <v>9</v>
+      </c>
+      <c r="V183" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n">
@@ -13700,6 +14802,12 @@
         </is>
       </c>
       <c r="T184" t="inlineStr"/>
+      <c r="U184" t="n">
+        <v>9</v>
+      </c>
+      <c r="V184" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="n">
@@ -13772,6 +14880,12 @@
         </is>
       </c>
       <c r="T185" t="inlineStr"/>
+      <c r="U185" t="n">
+        <v>9</v>
+      </c>
+      <c r="V185" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="n">
@@ -13844,6 +14958,12 @@
         </is>
       </c>
       <c r="T186" t="inlineStr"/>
+      <c r="U186" t="n">
+        <v>9</v>
+      </c>
+      <c r="V186" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n">
@@ -13916,6 +15036,12 @@
         </is>
       </c>
       <c r="T187" t="inlineStr"/>
+      <c r="U187" t="n">
+        <v>9</v>
+      </c>
+      <c r="V187" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n">
@@ -13988,6 +15114,12 @@
         </is>
       </c>
       <c r="T188" t="inlineStr"/>
+      <c r="U188" t="n">
+        <v>9</v>
+      </c>
+      <c r="V188" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n">
@@ -14060,6 +15192,12 @@
         </is>
       </c>
       <c r="T189" t="inlineStr"/>
+      <c r="U189" t="n">
+        <v>9</v>
+      </c>
+      <c r="V189" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
@@ -14132,6 +15270,12 @@
         </is>
       </c>
       <c r="T190" t="inlineStr"/>
+      <c r="U190" t="n">
+        <v>9</v>
+      </c>
+      <c r="V190" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n">
@@ -14204,6 +15348,12 @@
         </is>
       </c>
       <c r="T191" t="inlineStr"/>
+      <c r="U191" t="n">
+        <v>9</v>
+      </c>
+      <c r="V191" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="n">
@@ -14276,6 +15426,12 @@
         </is>
       </c>
       <c r="T192" t="inlineStr"/>
+      <c r="U192" t="n">
+        <v>9</v>
+      </c>
+      <c r="V192" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="n">
@@ -14348,6 +15504,12 @@
         </is>
       </c>
       <c r="T193" t="inlineStr"/>
+      <c r="U193" t="n">
+        <v>9</v>
+      </c>
+      <c r="V193" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="n">
@@ -14420,6 +15582,12 @@
         </is>
       </c>
       <c r="T194" t="inlineStr"/>
+      <c r="U194" t="n">
+        <v>9</v>
+      </c>
+      <c r="V194" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n">
@@ -14492,6 +15660,12 @@
         </is>
       </c>
       <c r="T195" t="inlineStr"/>
+      <c r="U195" t="n">
+        <v>9</v>
+      </c>
+      <c r="V195" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="n">
@@ -14564,6 +15738,12 @@
         </is>
       </c>
       <c r="T196" t="inlineStr"/>
+      <c r="U196" t="n">
+        <v>9</v>
+      </c>
+      <c r="V196" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="n">
@@ -14636,6 +15816,12 @@
         </is>
       </c>
       <c r="T197" t="inlineStr"/>
+      <c r="U197" t="n">
+        <v>9</v>
+      </c>
+      <c r="V197" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="n">
@@ -14708,6 +15894,12 @@
         </is>
       </c>
       <c r="T198" t="inlineStr"/>
+      <c r="U198" t="n">
+        <v>9</v>
+      </c>
+      <c r="V198" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="n">
@@ -14780,6 +15972,12 @@
         </is>
       </c>
       <c r="T199" t="inlineStr"/>
+      <c r="U199" t="n">
+        <v>9</v>
+      </c>
+      <c r="V199" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="n">
@@ -14852,6 +16050,12 @@
         </is>
       </c>
       <c r="T200" t="inlineStr"/>
+      <c r="U200" t="n">
+        <v>9</v>
+      </c>
+      <c r="V200" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="n">
@@ -14924,6 +16128,12 @@
         </is>
       </c>
       <c r="T201" t="inlineStr"/>
+      <c r="U201" t="n">
+        <v>9</v>
+      </c>
+      <c r="V201" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="n">
@@ -14996,6 +16206,12 @@
         </is>
       </c>
       <c r="T202" t="inlineStr"/>
+      <c r="U202" t="n">
+        <v>9</v>
+      </c>
+      <c r="V202" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="n">
@@ -15068,6 +16284,12 @@
         </is>
       </c>
       <c r="T203" t="inlineStr"/>
+      <c r="U203" t="n">
+        <v>9</v>
+      </c>
+      <c r="V203" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="n">
@@ -15140,6 +16362,12 @@
         </is>
       </c>
       <c r="T204" t="inlineStr"/>
+      <c r="U204" t="n">
+        <v>9</v>
+      </c>
+      <c r="V204" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="n">
@@ -15212,6 +16440,12 @@
         </is>
       </c>
       <c r="T205" t="inlineStr"/>
+      <c r="U205" t="n">
+        <v>9</v>
+      </c>
+      <c r="V205" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
@@ -15284,6 +16518,12 @@
         </is>
       </c>
       <c r="T206" t="inlineStr"/>
+      <c r="U206" t="n">
+        <v>9</v>
+      </c>
+      <c r="V206" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="n">
@@ -15356,6 +16596,12 @@
         </is>
       </c>
       <c r="T207" t="inlineStr"/>
+      <c r="U207" t="n">
+        <v>9</v>
+      </c>
+      <c r="V207" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="n">
@@ -15428,6 +16674,12 @@
         </is>
       </c>
       <c r="T208" t="inlineStr"/>
+      <c r="U208" t="n">
+        <v>9</v>
+      </c>
+      <c r="V208" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="n">
@@ -15500,6 +16752,12 @@
         </is>
       </c>
       <c r="T209" t="inlineStr"/>
+      <c r="U209" t="n">
+        <v>9</v>
+      </c>
+      <c r="V209" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="n">
@@ -15572,6 +16830,12 @@
         </is>
       </c>
       <c r="T210" t="inlineStr"/>
+      <c r="U210" t="n">
+        <v>9</v>
+      </c>
+      <c r="V210" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="n">
@@ -15644,6 +16908,12 @@
         </is>
       </c>
       <c r="T211" t="inlineStr"/>
+      <c r="U211" t="n">
+        <v>9</v>
+      </c>
+      <c r="V211" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="n">
@@ -15716,6 +16986,12 @@
         </is>
       </c>
       <c r="T212" t="inlineStr"/>
+      <c r="U212" t="n">
+        <v>9</v>
+      </c>
+      <c r="V212" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="n">
@@ -15788,6 +17064,12 @@
         </is>
       </c>
       <c r="T213" t="inlineStr"/>
+      <c r="U213" t="n">
+        <v>9</v>
+      </c>
+      <c r="V213" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="n">
@@ -15860,6 +17142,12 @@
         </is>
       </c>
       <c r="T214" t="inlineStr"/>
+      <c r="U214" t="n">
+        <v>9</v>
+      </c>
+      <c r="V214" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
@@ -15932,6 +17220,12 @@
         </is>
       </c>
       <c r="T215" t="inlineStr"/>
+      <c r="U215" t="n">
+        <v>9</v>
+      </c>
+      <c r="V215" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="n">
@@ -16004,6 +17298,12 @@
         </is>
       </c>
       <c r="T216" t="inlineStr"/>
+      <c r="U216" t="n">
+        <v>9</v>
+      </c>
+      <c r="V216" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="n">
@@ -16076,6 +17376,12 @@
         </is>
       </c>
       <c r="T217" t="inlineStr"/>
+      <c r="U217" t="n">
+        <v>9</v>
+      </c>
+      <c r="V217" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="n">
@@ -16148,6 +17454,12 @@
         </is>
       </c>
       <c r="T218" t="inlineStr"/>
+      <c r="U218" t="n">
+        <v>9</v>
+      </c>
+      <c r="V218" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="n">
@@ -16220,6 +17532,12 @@
         </is>
       </c>
       <c r="T219" t="inlineStr"/>
+      <c r="U219" t="n">
+        <v>9</v>
+      </c>
+      <c r="V219" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="n">
@@ -16292,6 +17610,12 @@
         </is>
       </c>
       <c r="T220" t="inlineStr"/>
+      <c r="U220" t="n">
+        <v>9</v>
+      </c>
+      <c r="V220" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="n">
@@ -16364,6 +17688,12 @@
         </is>
       </c>
       <c r="T221" t="inlineStr"/>
+      <c r="U221" t="n">
+        <v>9</v>
+      </c>
+      <c r="V221" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="n">
@@ -16436,6 +17766,12 @@
         </is>
       </c>
       <c r="T222" t="inlineStr"/>
+      <c r="U222" t="n">
+        <v>9</v>
+      </c>
+      <c r="V222" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n">
@@ -16508,6 +17844,12 @@
         </is>
       </c>
       <c r="T223" t="inlineStr"/>
+      <c r="U223" t="n">
+        <v>9</v>
+      </c>
+      <c r="V223" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="n">
@@ -16580,6 +17922,12 @@
         </is>
       </c>
       <c r="T224" t="inlineStr"/>
+      <c r="U224" t="n">
+        <v>9</v>
+      </c>
+      <c r="V224" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="n">
@@ -16652,6 +18000,12 @@
         </is>
       </c>
       <c r="T225" t="inlineStr"/>
+      <c r="U225" t="n">
+        <v>9</v>
+      </c>
+      <c r="V225" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="n">
@@ -16724,6 +18078,12 @@
         </is>
       </c>
       <c r="T226" t="inlineStr"/>
+      <c r="U226" t="n">
+        <v>9</v>
+      </c>
+      <c r="V226" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="n">
@@ -16796,6 +18156,12 @@
         </is>
       </c>
       <c r="T227" t="inlineStr"/>
+      <c r="U227" t="n">
+        <v>9</v>
+      </c>
+      <c r="V227" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="n">
@@ -16868,6 +18234,12 @@
         </is>
       </c>
       <c r="T228" t="inlineStr"/>
+      <c r="U228" t="n">
+        <v>9</v>
+      </c>
+      <c r="V228" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="n">
@@ -16940,6 +18312,12 @@
         </is>
       </c>
       <c r="T229" t="inlineStr"/>
+      <c r="U229" t="n">
+        <v>9</v>
+      </c>
+      <c r="V229" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="n">
@@ -17012,6 +18390,12 @@
         </is>
       </c>
       <c r="T230" t="inlineStr"/>
+      <c r="U230" t="n">
+        <v>9</v>
+      </c>
+      <c r="V230" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="n">
@@ -17084,6 +18468,12 @@
         </is>
       </c>
       <c r="T231" t="inlineStr"/>
+      <c r="U231" t="n">
+        <v>9</v>
+      </c>
+      <c r="V231" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="n">
@@ -17156,6 +18546,12 @@
         </is>
       </c>
       <c r="T232" t="inlineStr"/>
+      <c r="U232" t="n">
+        <v>9</v>
+      </c>
+      <c r="V232" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="n">
@@ -17228,6 +18624,12 @@
         </is>
       </c>
       <c r="T233" t="inlineStr"/>
+      <c r="U233" t="n">
+        <v>9</v>
+      </c>
+      <c r="V233" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="n">
@@ -17300,6 +18702,12 @@
         </is>
       </c>
       <c r="T234" t="inlineStr"/>
+      <c r="U234" t="n">
+        <v>9</v>
+      </c>
+      <c r="V234" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="n">
@@ -17372,6 +18780,12 @@
         </is>
       </c>
       <c r="T235" t="inlineStr"/>
+      <c r="U235" t="n">
+        <v>9</v>
+      </c>
+      <c r="V235" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="n">
@@ -17444,6 +18858,12 @@
         </is>
       </c>
       <c r="T236" t="inlineStr"/>
+      <c r="U236" t="n">
+        <v>9</v>
+      </c>
+      <c r="V236" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="n">
@@ -17516,6 +18936,12 @@
         </is>
       </c>
       <c r="T237" t="inlineStr"/>
+      <c r="U237" t="n">
+        <v>9</v>
+      </c>
+      <c r="V237" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="n">
@@ -17588,6 +19014,12 @@
         </is>
       </c>
       <c r="T238" t="inlineStr"/>
+      <c r="U238" t="n">
+        <v>9</v>
+      </c>
+      <c r="V238" t="n">
+        <v>54</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="n">
@@ -17660,6 +19092,12 @@
         </is>
       </c>
       <c r="T239" t="inlineStr"/>
+      <c r="U239" t="n">
+        <v>9</v>
+      </c>
+      <c r="V239" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="n">
@@ -17732,6 +19170,12 @@
         </is>
       </c>
       <c r="T240" t="inlineStr"/>
+      <c r="U240" t="n">
+        <v>9</v>
+      </c>
+      <c r="V240" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="n">
@@ -17804,6 +19248,12 @@
         </is>
       </c>
       <c r="T241" t="inlineStr"/>
+      <c r="U241" t="n">
+        <v>9</v>
+      </c>
+      <c r="V241" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="n">
@@ -17876,6 +19326,12 @@
         </is>
       </c>
       <c r="T242" t="inlineStr"/>
+      <c r="U242" t="n">
+        <v>9</v>
+      </c>
+      <c r="V242" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="n">
@@ -17948,6 +19404,12 @@
         </is>
       </c>
       <c r="T243" t="inlineStr"/>
+      <c r="U243" t="n">
+        <v>9</v>
+      </c>
+      <c r="V243" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="n">
@@ -18020,6 +19482,12 @@
         </is>
       </c>
       <c r="T244" t="inlineStr"/>
+      <c r="U244" t="n">
+        <v>9</v>
+      </c>
+      <c r="V244" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
@@ -18092,6 +19560,12 @@
         </is>
       </c>
       <c r="T245" t="inlineStr"/>
+      <c r="U245" t="n">
+        <v>9</v>
+      </c>
+      <c r="V245" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="n">
@@ -18164,6 +19638,12 @@
         </is>
       </c>
       <c r="T246" t="inlineStr"/>
+      <c r="U246" t="n">
+        <v>9</v>
+      </c>
+      <c r="V246" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="n">
@@ -18236,6 +19716,12 @@
         </is>
       </c>
       <c r="T247" t="inlineStr"/>
+      <c r="U247" t="n">
+        <v>9</v>
+      </c>
+      <c r="V247" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="n">
@@ -18308,6 +19794,12 @@
         </is>
       </c>
       <c r="T248" t="inlineStr"/>
+      <c r="U248" t="n">
+        <v>9</v>
+      </c>
+      <c r="V248" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="n">
@@ -18380,6 +19872,12 @@
         </is>
       </c>
       <c r="T249" t="inlineStr"/>
+      <c r="U249" t="n">
+        <v>9</v>
+      </c>
+      <c r="V249" t="n">
+        <v>49</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>